<commit_message>
feat(combat): G01-P7-M01 implement Assist skill subsystem
</commit_message>
<xml_diff>
--- a/config/generated/templates/Ability.xlsx
+++ b/config/generated/templates/Ability.xlsx
@@ -43,7 +43,7 @@
     <t>@schema</t>
   </si>
   <si>
-    <t>e585469aa7aa7a4a</t>
+    <t>8bed349bb757ef1d</t>
   </si>
   <si>
     <t>#name</t>
@@ -109,7 +109,7 @@
     <t>range=0..100</t>
   </si>
   <si>
-    <t>range=0..2047</t>
+    <t>range=0..4095</t>
   </si>
   <si>
     <t>#desc</t>
@@ -744,9 +744,9 @@
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 0 to 2047." promptTitle="Integer range" prompt="Enter an integer from 0 to 2047." sqref="H8:H1007">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 0 to 4095." promptTitle="Integer range" prompt="Enter an integer from 0 to 4095." sqref="H8:H1007">
       <formula1>0</formula1>
-      <formula2>2047</formula2>
+      <formula2>4095</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>